<commit_message>
fix(wifi_llapi): 以投影 bucket 統計 Summary fail
保留 Wifi_LLAPI raw verdict，新增隱藏 summary bucket 欄位供 Summary 公式統計，避免 env/setup/counter 類非 pass criteria fail 被算入 Fail。

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/plugins/wifi_llapi/reports/templates/wifi_llapi_template.xlsx
+++ b/plugins/wifi_llapi/reports/templates/wifi_llapi_template.xlsx
@@ -1826,23 +1826,23 @@
         <v/>
       </c>
       <c r="E3" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$I:$I,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$N:$N,E$2)</f>
         <v/>
       </c>
       <c r="F3" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$I:$I,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$N:$N,F$2)</f>
         <v/>
       </c>
       <c r="G3" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$I:$I,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$N:$N,G$2)</f>
         <v/>
       </c>
       <c r="H3" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$I:$I,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$I:$I,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$N:$N,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$N:$N,"")</f>
         <v/>
       </c>
       <c r="I3" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$I:$I,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$I:$I,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$N:$N,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B3&amp;"*",Wifi_LLAPI!$N:$N,"N/A")</f>
         <v/>
       </c>
       <c r="J3" s="155">
@@ -1889,23 +1889,23 @@
         <v/>
       </c>
       <c r="E4" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$I:$I,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$N:$N,E$2)</f>
         <v/>
       </c>
       <c r="F4" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$I:$I,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$N:$N,F$2)</f>
         <v/>
       </c>
       <c r="G4" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$I:$I,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$N:$N,G$2)</f>
         <v/>
       </c>
       <c r="H4" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$I:$I,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$I:$I,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$N:$N,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$N:$N,"")</f>
         <v/>
       </c>
       <c r="I4" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$I:$I,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$I:$I,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$N:$N,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B4&amp;"*",Wifi_LLAPI!$N:$N,"N/A")</f>
         <v/>
       </c>
       <c r="J4" s="150">
@@ -1949,23 +1949,23 @@
         <v/>
       </c>
       <c r="E5" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$I:$I,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$N:$N,E$2)</f>
         <v/>
       </c>
       <c r="F5" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$I:$I,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$N:$N,F$2)</f>
         <v/>
       </c>
       <c r="G5" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$I:$I,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$N:$N,G$2)</f>
         <v/>
       </c>
       <c r="H5" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$I:$I,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$I:$I,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$N:$N,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$N:$N,"")</f>
         <v/>
       </c>
       <c r="I5" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$I:$I,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$I:$I,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$N:$N,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B5&amp;"*",Wifi_LLAPI!$N:$N,"N/A")</f>
         <v/>
       </c>
       <c r="J5" s="150">
@@ -2009,23 +2009,23 @@
         <v/>
       </c>
       <c r="E6" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$I:$I,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$N:$N,E$2)</f>
         <v/>
       </c>
       <c r="F6" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$I:$I,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$N:$N,F$2)</f>
         <v/>
       </c>
       <c r="G6" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$I:$I,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$N:$N,G$2)</f>
         <v/>
       </c>
       <c r="H6" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$I:$I,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$I:$I,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$N:$N,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$N:$N,"")</f>
         <v/>
       </c>
       <c r="I6" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$I:$I,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$I:$I,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$N:$N,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B6&amp;"*",Wifi_LLAPI!$N:$N,"N/A")</f>
         <v/>
       </c>
       <c r="J6" s="150">
@@ -2069,23 +2069,23 @@
         <v/>
       </c>
       <c r="E7" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$I:$I,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$N:$N,E$2)</f>
         <v/>
       </c>
       <c r="F7" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$I:$I,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$N:$N,F$2)</f>
         <v/>
       </c>
       <c r="G7" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$I:$I,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$N:$N,G$2)</f>
         <v/>
       </c>
       <c r="H7" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$I:$I,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$I:$I,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$N:$N,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$N:$N,"")</f>
         <v/>
       </c>
       <c r="I7" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$I:$I,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$I:$I,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$N:$N,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B7&amp;"*",Wifi_LLAPI!$N:$N,"N/A")</f>
         <v/>
       </c>
       <c r="J7" s="150">
@@ -2169,23 +2169,23 @@
         <v/>
       </c>
       <c r="E9" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$J:$J,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$O:$O,E$2)</f>
         <v/>
       </c>
       <c r="F9" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$J:$J,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$O:$O,F$2)</f>
         <v/>
       </c>
       <c r="G9" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$J:$J,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$O:$O,G$2)</f>
         <v/>
       </c>
       <c r="H9" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$J:$J,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$J:$J,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$O:$O,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$O:$O,"")</f>
         <v/>
       </c>
       <c r="I9" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$J:$J,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$J:$J,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$O:$O,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B9&amp;"*",Wifi_LLAPI!$O:$O,"N/A")</f>
         <v/>
       </c>
       <c r="J9" s="155">
@@ -2217,23 +2217,23 @@
         <v/>
       </c>
       <c r="E10" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$J:$J,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$O:$O,E$2)</f>
         <v/>
       </c>
       <c r="F10" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$J:$J,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$O:$O,F$2)</f>
         <v/>
       </c>
       <c r="G10" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$J:$J,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$O:$O,G$2)</f>
         <v/>
       </c>
       <c r="H10" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$J:$J,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$J:$J,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$O:$O,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$O:$O,"")</f>
         <v/>
       </c>
       <c r="I10" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$J:$J,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$J:$J,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$O:$O,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B10&amp;"*",Wifi_LLAPI!$O:$O,"N/A")</f>
         <v/>
       </c>
       <c r="J10" s="150">
@@ -2265,23 +2265,23 @@
         <v/>
       </c>
       <c r="E11" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$J:$J,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$O:$O,E$2)</f>
         <v/>
       </c>
       <c r="F11" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$J:$J,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$O:$O,F$2)</f>
         <v/>
       </c>
       <c r="G11" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$J:$J,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$O:$O,G$2)</f>
         <v/>
       </c>
       <c r="H11" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$J:$J,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$J:$J,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$O:$O,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$O:$O,"")</f>
         <v/>
       </c>
       <c r="I11" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$J:$J,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$J:$J,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$O:$O,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B11&amp;"*",Wifi_LLAPI!$O:$O,"N/A")</f>
         <v/>
       </c>
       <c r="J11" s="150">
@@ -2313,23 +2313,23 @@
         <v/>
       </c>
       <c r="E12" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$J:$J,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$O:$O,E$2)</f>
         <v/>
       </c>
       <c r="F12" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$J:$J,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$O:$O,F$2)</f>
         <v/>
       </c>
       <c r="G12" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$J:$J,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$O:$O,G$2)</f>
         <v/>
       </c>
       <c r="H12" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$J:$J,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$J:$J,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$O:$O,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$O:$O,"")</f>
         <v/>
       </c>
       <c r="I12" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$J:$J,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$J:$J,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$O:$O,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B12&amp;"*",Wifi_LLAPI!$O:$O,"N/A")</f>
         <v/>
       </c>
       <c r="J12" s="150">
@@ -2361,23 +2361,23 @@
         <v/>
       </c>
       <c r="E13" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$J:$J,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$O:$O,E$2)</f>
         <v/>
       </c>
       <c r="F13" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$J:$J,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$O:$O,F$2)</f>
         <v/>
       </c>
       <c r="G13" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$J:$J,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$O:$O,G$2)</f>
         <v/>
       </c>
       <c r="H13" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$J:$J,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$J:$J,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$O:$O,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$O:$O,"")</f>
         <v/>
       </c>
       <c r="I13" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$J:$J,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$J:$J,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$O:$O,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B13&amp;"*",Wifi_LLAPI!$O:$O,"N/A")</f>
         <v/>
       </c>
       <c r="J13" s="150">
@@ -2461,23 +2461,23 @@
         <v/>
       </c>
       <c r="E15" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$K:$K,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$P:$P,E$2)</f>
         <v/>
       </c>
       <c r="F15" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$K:$K,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$P:$P,F$2)</f>
         <v/>
       </c>
       <c r="G15" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$K:$K,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$P:$P,G$2)</f>
         <v/>
       </c>
       <c r="H15" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$K:$K,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$K:$K,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$P:$P,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$P:$P,"")</f>
         <v/>
       </c>
       <c r="I15" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$K:$K,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$K:$K,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$P:$P,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B15&amp;"*",Wifi_LLAPI!$P:$P,"N/A")</f>
         <v/>
       </c>
       <c r="J15" s="155">
@@ -2509,23 +2509,23 @@
         <v/>
       </c>
       <c r="E16" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$K:$K,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$P:$P,E$2)</f>
         <v/>
       </c>
       <c r="F16" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$K:$K,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$P:$P,F$2)</f>
         <v/>
       </c>
       <c r="G16" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$K:$K,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$P:$P,G$2)</f>
         <v/>
       </c>
       <c r="H16" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$K:$K,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$K:$K,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$P:$P,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$P:$P,"")</f>
         <v/>
       </c>
       <c r="I16" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$K:$K,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$K:$K,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$P:$P,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B16&amp;"*",Wifi_LLAPI!$P:$P,"N/A")</f>
         <v/>
       </c>
       <c r="J16" s="150">
@@ -2557,23 +2557,23 @@
         <v/>
       </c>
       <c r="E17" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$K:$K,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$P:$P,E$2)</f>
         <v/>
       </c>
       <c r="F17" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$K:$K,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$P:$P,F$2)</f>
         <v/>
       </c>
       <c r="G17" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$K:$K,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$P:$P,G$2)</f>
         <v/>
       </c>
       <c r="H17" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$K:$K,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$K:$K,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$P:$P,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$P:$P,"")</f>
         <v/>
       </c>
       <c r="I17" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$K:$K,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$K:$K,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$P:$P,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B17&amp;"*",Wifi_LLAPI!$P:$P,"N/A")</f>
         <v/>
       </c>
       <c r="J17" s="150">
@@ -2605,23 +2605,23 @@
         <v/>
       </c>
       <c r="E18" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$K:$K,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$P:$P,E$2)</f>
         <v/>
       </c>
       <c r="F18" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$K:$K,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$P:$P,F$2)</f>
         <v/>
       </c>
       <c r="G18" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$K:$K,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$P:$P,G$2)</f>
         <v/>
       </c>
       <c r="H18" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$K:$K,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$K:$K,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$P:$P,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$P:$P,"")</f>
         <v/>
       </c>
       <c r="I18" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$K:$K,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$K:$K,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$P:$P,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B18&amp;"*",Wifi_LLAPI!$P:$P,"N/A")</f>
         <v/>
       </c>
       <c r="J18" s="150">
@@ -2653,23 +2653,23 @@
         <v/>
       </c>
       <c r="E19" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$K:$K,E$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$P:$P,E$2)</f>
         <v/>
       </c>
       <c r="F19" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$K:$K,F$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$P:$P,F$2)</f>
         <v/>
       </c>
       <c r="G19" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$K:$K,G$2)</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$P:$P,G$2)</f>
         <v/>
       </c>
       <c r="H19" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$K:$K,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$K:$K,"")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$P:$P,H$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$E:$E,"Not Supported",Wifi_LLAPI!$P:$P,"")</f>
         <v/>
       </c>
       <c r="I19" s="151">
-        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$K:$K,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$K:$K,"N/A")</f>
+        <f>COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$P:$P,I$2)+COUNTIFS(Wifi_LLAPI!$A:$A,$B19&amp;"*",Wifi_LLAPI!$P:$P,"N/A")</f>
         <v/>
       </c>
       <c r="J19" s="150">
@@ -2789,7 +2789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M573715"/>
+  <dimension ref="A1:P573715"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9.875" customWidth="1" style="18" min="1" max="1"/>
@@ -2800,6 +2800,9 @@
     <col width="25.625" bestFit="1" customWidth="1" style="20" min="7" max="7"/>
     <col width="9" customWidth="1" style="21" min="8" max="8"/>
     <col width="9" customWidth="1" style="22" min="9" max="12"/>
+    <col hidden="1" width="13" customWidth="1" style="180" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" style="180" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" style="180" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="33.75" customHeight="1" s="180">
@@ -2963,6 +2966,21 @@
       <c r="M3" s="122" t="inlineStr">
         <is>
           <t>Comment</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Summary Bucket WiFi 5G</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Summary Bucket WiFi 6G</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Summary Bucket WiFi 2.4G</t>
         </is>
       </c>
     </row>

</xml_diff>